<commit_message>
fix: close v6.15.9 live audit findings (v6.15.10)
</commit_message>
<xml_diff>
--- a/resources/templates/Template_TaxTool_FS_AI.xlsx
+++ b/resources/templates/Template_TaxTool_FS_AI.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="Re12f2f6ec3694db5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="R8a493d7f20054505"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voci IV Direttiva" sheetId="3" r:id="Rc2b6b78cb9344054"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stato Patrimoniale" sheetId="4" r:id="R4288c6669e6349ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conto Economico" sheetId="5" r:id="R54350bac1d774681"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esiti AI" sheetId="6" r:id="R6d17dd59a07b4258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="1" r:id="R54b8cc3323e34edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Anagrafica" sheetId="2" r:id="Rb894d93179b04956"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Voci IV Direttiva" sheetId="3" r:id="Rede716fbdd104b07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stato Patrimoniale" sheetId="4" r:id="Reb3ca8838bf146e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conto Economico" sheetId="5" r:id="R5a88d668becc481c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esiti AI" sheetId="6" r:id="R049b93ebe3ff4c07"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -256,7 +256,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="2" t="str">
-        <x:v>TAX AUTOMATION LAB — RICLASSIFICA IV DIRETTIVA v1.3.5</x:v>
+        <x:v>TAX AUTOMATION LAB — RICLASSIFICA IV DIRETTIVA v1.3.6</x:v>
       </x:c>
     </x:row>
     <x:row r="2">

</xml_diff>